<commit_message>
Finalisation module menages - saisie M04 cout complet
</commit_message>
<xml_diff>
--- a/01_SOURCES_BRUTES/Charges/SAISIE_Charges_Flux.xlsx
+++ b/01_SOURCES_BRUTES/Charges/SAISIE_Charges_Flux.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="SAISIE" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="REF_LOCALE" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="CONTROLES_SAISIE" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="README" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAISIE" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REF_LOCALE" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONTROLES_SAISIE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="lst_Categories">'REF_LOCALE'!$A$2:$A$24</definedName>
@@ -273,6 +273,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>lot6</author>
+  </authors>
+  <commentList>
+    <comment ref="AG1" authorId="0" shapeId="0">
+      <text>
+        <t>Valeurs: MENAGE_INTERNE / COMMUN_MENAGE / INT_xxxx / INT_xxxx;INT_yyyy (séparateur ;)</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -564,7 +579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE501"/>
+  <dimension ref="A1:AG501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -756,6 +771,16 @@
           <t>date_saisie</t>
         </is>
       </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>affectable_menage</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>intervenant_concerne</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="C2">
@@ -9766,7 +9791,7 @@
       <formula>$Y2="A_CONTROLER"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="18">
+  <dataValidations count="19">
     <dataValidation sqref="E2:E1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur invalide" error="Valeur hors liste. Utiliser la liste deroulante." type="list">
       <formula1>lst_Sens_Flux</formula1>
     </dataValidation>
@@ -9821,8 +9846,12 @@
     <dataValidation sqref="AB2:AB1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur invalide" error="Valeur hors liste. Utiliser la liste deroulante." type="list">
       <formula1>lst_Justificatif</formula1>
     </dataValidation>
+    <dataValidation sqref="AF2:AF501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Valeurs: OUI / NON / A_CONTROLER" prompt="OUI=affecté ménages, NON=ignoré, A_CONTROLER" type="list">
+      <formula1>"OUI,NON,A_CONTROLER"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -10606,7 +10635,6 @@
           <t>INFO</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -10628,7 +10656,6 @@
           <t>INFO</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -10650,7 +10677,6 @@
           <t>ATTENTION si &gt; 0</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10672,7 +10698,6 @@
           <t>INFO</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -10694,7 +10719,6 @@
           <t>ATTENTION si &gt; 0</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -10768,7 +10792,6 @@
           <t>INFO</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -10790,7 +10813,6 @@
           <t>INFO</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -10864,7 +10886,6 @@
           <t>BLOQUANT si &gt; 0</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">

</xml_diff>

<commit_message>
Référentiel : profils impact et catégorie personnalisée
</commit_message>
<xml_diff>
--- a/01_SOURCES_BRUTES/Charges/SAISIE_Charges_Flux.xlsx
+++ b/01_SOURCES_BRUTES/Charges/SAISIE_Charges_Flux.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="lst_Categories">'REF_LOCALE'!$A$2:$A$24</definedName>
+    <definedName name="lst_Categories">'REF_LOCALE'!$A$2:$A$25</definedName>
     <definedName name="lst_TypesFlux_Lot3">'REF_LOCALE'!$B$2:$B$8</definedName>
     <definedName name="lst_Codes_Impact">'REF_LOCALE'!$C$2:$C$4</definedName>
     <definedName name="lst_Sens_Flux">'REF_LOCALE'!$D$2:$D$6</definedName>
@@ -31,6 +31,7 @@
     <definedName name="lst_Prise_Compta">'REF_LOCALE'!$P$2:$P$3</definedName>
     <definedName name="lst_Refacturable">'REF_LOCALE'!$Q$2:$Q$3</definedName>
     <definedName name="lst_Justificatif">'REF_LOCALE'!$R$2:$R$4</definedName>
+    <definedName name="lst_Profils_Impact">'REF_LOCALE'!$S$2:$S$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -579,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG501"/>
+  <dimension ref="A1:AI501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -781,6 +782,16 @@
           <t>intervenant_concerne</t>
         </is>
       </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>profil_impact_charge</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>libelle_categorie_personnalise</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="C2">
@@ -9791,7 +9802,7 @@
       <formula>$Y2="A_CONTROLER"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="19">
+  <dataValidations count="20">
     <dataValidation sqref="E2:E1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur invalide" error="Valeur hors liste. Utiliser la liste deroulante." type="list">
       <formula1>lst_Sens_Flux</formula1>
     </dataValidation>
@@ -9849,6 +9860,9 @@
     <dataValidation sqref="AF2:AF501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Valeurs: OUI / NON / A_CONTROLER" prompt="OUI=affecté ménages, NON=ignoré, A_CONTROLER" type="list">
       <formula1>"OUI,NON,A_CONTROLER"</formula1>
     </dataValidation>
+    <dataValidation sqref="AH2:AH1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>lst_Profils_Impact</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -9861,7 +9875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R24"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -9975,6 +9989,11 @@
           <t>lst_Justificatif</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>lst_Profils_Impact</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -10067,6 +10086,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -10159,6 +10183,11 @@
           <t>NON</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>LOGEMENT_DIRECT</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -10231,6 +10260,11 @@
           <t>LIEN</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>MENAGE_INTERVENANT</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10288,6 +10322,11 @@
           <t>ECART_A_ANALYSER</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>MENAGE_LOGEMENTS</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -10330,6 +10369,11 @@
           <t>A_CONFIRMER</t>
         </is>
       </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>PARCOURS_DEDIE</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -10564,6 +10608,13 @@
       <c r="A24" t="inlineStr">
         <is>
           <t>CHG_023</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CHG_024</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Référentiel : types flux et parcours dédiés charges
</commit_message>
<xml_diff>
--- a/01_SOURCES_BRUTES/Charges/SAISIE_Charges_Flux.xlsx
+++ b/01_SOURCES_BRUTES/Charges/SAISIE_Charges_Flux.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="lst_Categories">'REF_LOCALE'!$A$2:$A$25</definedName>
-    <definedName name="lst_TypesFlux_Lot3">'REF_LOCALE'!$B$2:$B$8</definedName>
+    <definedName name="lst_TypesFlux_Lot3">'REF_LOCALE'!$B$2:$B$10</definedName>
     <definedName name="lst_Codes_Impact">'REF_LOCALE'!$C$2:$C$4</definedName>
     <definedName name="lst_Sens_Flux">'REF_LOCALE'!$D$2:$D$6</definedName>
     <definedName name="lst_Associes">'REF_LOCALE'!$E$2:$E$3</definedName>
@@ -10425,6 +10425,11 @@
           <t>CHG_008</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TYPE_FLUX_016</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>LOG_0009</t>
@@ -10440,6 +10445,11 @@
       <c r="A10" t="inlineStr">
         <is>
           <t>CHG_009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TYPE_FLUX_020</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">

</xml_diff>

<commit_message>
Référentiel : catégories Nouvelle charge (repas, prestation, supplément ménage)
</commit_message>
<xml_diff>
--- a/01_SOURCES_BRUTES/Charges/SAISIE_Charges_Flux.xlsx
+++ b/01_SOURCES_BRUTES/Charges/SAISIE_Charges_Flux.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="lst_Categories">'REF_LOCALE'!$A$2:$A$25</definedName>
+    <definedName name="lst_Categories">'REF_LOCALE'!$A$2:$A$28</definedName>
     <definedName name="lst_TypesFlux_Lot3">'REF_LOCALE'!$B$2:$B$10</definedName>
     <definedName name="lst_Codes_Impact">'REF_LOCALE'!$C$2:$C$4</definedName>
     <definedName name="lst_Sens_Flux">'REF_LOCALE'!$D$2:$D$6</definedName>
@@ -9875,7 +9875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S25"/>
+  <dimension ref="A1:S28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10628,6 +10628,27 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CHG_025</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CHG_026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CHG_027</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Avantage porté par la charge + Lot7 lib agrégation (anti double comptage)
</commit_message>
<xml_diff>
--- a/01_SOURCES_BRUTES/Charges/SAISIE_Charges_Flux.xlsx
+++ b/01_SOURCES_BRUTES/Charges/SAISIE_Charges_Flux.xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI501"/>
+  <dimension ref="A1:AJ501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -790,6 +790,11 @@
       <c r="AI1" t="inlineStr">
         <is>
           <t>libelle_categorie_personnalise</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>avantage_associe_id</t>
         </is>
       </c>
     </row>

</xml_diff>